<commit_message>
KiCad Power: charger, battery, 3.3 V LDO and fuel gauge
- Project symbol library Jot.kicad_sym with BQ25101, TPS7A0233 and
  MAX17048, pinouts taken from their datasheets
- Power sheet: BQ25101 charger (680R ISET ~200 mA, 10k TS), charge LED,
  battery connector, TPS7A0233 3.3 V LDO (EN tied to IN), MAX17048 fuel
  gauge on I2C with FG_ALRT, input/output caps, PWR_FLAGs on VBUS/GND
- Pin list net names now match KiCad power symbols (+BATT, +3V3, VBUS)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_Pin_List.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_Pin_List.xlsx
@@ -784,7 +784,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Q2 gate. LOW = mics + Rec LED on. 100k pull-up to 3V3.</t>
+          <t>Q2 gate. LOW = mics + Rec LED on. 100k pull-up to +3V3.</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>3V3</t>
+          <t>+3V3</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>3V3</t>
+          <t>+3V3</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -1496,7 +1496,7 @@
       <c r="E40" s="7" t="inlineStr"/>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Fuel gauge, accel, haptic driver. 4.7k pull-up to 3V3.</t>
+          <t>Fuel gauge, accel, haptic driver. 4.7k pull-up to +3V3.</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,7 @@
       <c r="E41" s="7" t="inlineStr"/>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Same bus. 4.7k pull-up to 3V3.</t>
+          <t>Same bus. 4.7k pull-up to +3V3.</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Use this when drawing the schematic: one row per net. Device pins are listed by name; check pin numbers in each footprint.</t>
+          <t>Use this when drawing the schematic: one row per net. Device pins are listed by name; check pin numbers in each footprint. Net names match the KiCad power symbols (+BATT, +3V3, VBUS, GND).</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>VBAT</t>
+          <t>+BATT</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>USB_VBUS</t>
+          <t>VBUS</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>R14 (2.2R from USB_VBUS), U1 VBUS (32), 10 uF to GND</t>
+          <t>R14 (2.2R from VBUS), U1 VBUS (32), 10 uF to GND</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>3V3</t>
+          <t>+3V3</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>U1 P0.13, U6 SDA, U7 SDA, U8 SDA, R3 (to 3V3)</t>
+          <t>U1 P0.13, U6 SDA, U7 SDA, U8 SDA, R3 (to +3V3)</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>U1 P0.14, U6 SCL, U7 SCL, U8 SCL, R4 (to 3V3)</t>
+          <t>U1 P0.14, U6 SCL, U7 SCL, U8 SCL, R4 (to +3V3)</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr"/>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>U1 P1.15, Q2 gate, R13 (to 3V3)</t>
+          <t>U1 P1.15, Q2 gate, R13 (to +3V3)</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>D3 anode via R11 to USB_VBUS.</t>
+          <t>D3 anode via R11 to VBUS.</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>Plus GND and 3V3 pads.</t>
+          <t>Plus GND and +3V3 pads.</t>
         </is>
       </c>
     </row>

</xml_diff>